<commit_message>
Non-initialized cell excluded from children of XLColumn and XLRow. Reference files updated (cells with default styles excluded)
</commit_message>
<xml_diff>
--- a/ClosedXML_Tests/Resource/Examples/Ranges/CurrentRowColumn.xlsx
+++ b/ClosedXML_Tests/Resource/Examples/Ranges/CurrentRowColumn.xlsx
@@ -438,7 +438,7 @@
   <x:sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14.020625" style="1" customWidth="1"/>
-    <x:col min="2" max="2" width="2.900625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="2.900625" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="9.140625" style="1" customWidth="1"/>
     <x:col min="4" max="4" width="15.970625" style="1" customWidth="1"/>
     <x:col min="5" max="5" width="2.900625" style="1" customWidth="1"/>
@@ -473,19 +473,13 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:5" s="0" customFormat="1">
-      <x:c r="A5" s="0" t="s"/>
+    <x:row r="5" spans="1:5">
       <x:c r="B5" s="2" t="s"/>
-      <x:c r="C5" s="0" t="s"/>
-      <x:c r="D5" s="0" t="s"/>
-      <x:c r="E5" s="0" t="s"/>
-    </x:row>
-    <x:row r="6" spans="1:5" s="0" customFormat="1">
+    </x:row>
+    <x:row r="6" spans="1:5">
       <x:c r="A6" s="3" t="s"/>
       <x:c r="B6" s="3" t="s"/>
       <x:c r="C6" s="3" t="s"/>
-      <x:c r="D6" s="0" t="s"/>
-      <x:c r="E6" s="0" t="s"/>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="B7" s="4" t="s"/>

</xml_diff>